<commit_message>
ng: update oncho forms
</commit_message>
<xml_diff>
--- a/ONCHO/Entomological survey Survey/Nigeria/2025/ng_oncho_2503_3_flies_sort_tar.xlsx
+++ b/ONCHO/Entomological survey Survey/Nigeria/2025/ng_oncho_2503_3_flies_sort_tar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\ONCHO\Entomological survey Survey\Nigeria\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2073EA-6A5C-4834-834E-30D945AF60EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DB157F-F32A-42A2-8486-634539F4D499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="248">
   <si>
     <t>type</t>
   </si>
@@ -185,9 +185,6 @@
   </si>
   <si>
     <t>Signature of State Coordinator</t>
-  </si>
-  <si>
-    <t>no</t>
   </si>
   <si>
     <t>January</t>
@@ -693,9 +690,6 @@
     <t>TAR_ARD_N_053</t>
   </si>
   <si>
-    <t>ng_oncho_2503_3_flies_sort_tar</t>
-  </si>
-  <si>
     <t>ZANGO KOBI</t>
   </si>
   <si>
@@ -747,14 +741,53 @@
     <t>TAR_SAR_N_053</t>
   </si>
   <si>
-    <t>(Taraba) 3. Blackfly Sorting Modules V4</t>
+    <t>ng_oncho_2503_3_flies_sort_tar_v4_2</t>
+  </si>
+  <si>
+    <t>(Taraba) 3. Blackfly Sorting Modules V4.2</t>
+  </si>
+  <si>
+    <t>.&lt;= 11</t>
+  </si>
+  <si>
+    <t>Days of collection must be less than or equal to 11</t>
+  </si>
+  <si>
+    <t>select_one yes_no</t>
+  </si>
+  <si>
+    <t>confirm_rec_zero_flies</t>
+  </si>
+  <si>
+    <t>You noted that 0 flies were collected for the month. Please confirm that collection took place and 0 flies were recorded.</t>
+  </si>
+  <si>
+    <t>. != 'No'</t>
+  </si>
+  <si>
+    <t>You entered there were zero flies, if that isn't the case, please update your previous answers accordingly.</t>
+  </si>
+  <si>
+    <t>${recorded_flies_both} = 0</t>
+  </si>
+  <si>
+    <t>confirm_zero_flies</t>
+  </si>
+  <si>
+    <t>You noted that 0 flies were morphologically confirmed for the month. Please confirm that sorting took place and 0 confirmed flies were recorded.</t>
+  </si>
+  <si>
+    <t>. != No</t>
+  </si>
+  <si>
+    <t>${total_num_confirmed_flies} = 0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -812,8 +845,21 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -850,8 +896,14 @@
         <bgColor rgb="FFCCFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -889,11 +941,71 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -956,6 +1068,27 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1310,7 +1443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:Y25"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.625" style="4" customWidth="1"/>
@@ -1329,7 +1462,7 @@
     <col min="14" max="16384" width="11" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="5" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" s="5" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1370,25 +1503,25 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>87</v>
       </c>
       <c r="E2" s="8"/>
       <c r="F2" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G2" s="10" t="s">
         <v>88</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>89</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
@@ -1398,15 +1531,15 @@
       <c r="K2" s="8"/>
       <c r="M2" s="8"/>
     </row>
-    <row r="3" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>96</v>
-      </c>
       <c r="C3" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="8"/>
@@ -1421,12 +1554,12 @@
       <c r="L3" s="8"/>
       <c r="M3" s="8"/>
     </row>
-    <row r="4" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>97</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>98</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>37</v>
@@ -1442,16 +1575,16 @@
       </c>
       <c r="K4" s="8"/>
       <c r="L4" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M4" s="8"/>
     </row>
-    <row r="5" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>100</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>38</v>
@@ -1467,19 +1600,19 @@
       </c>
       <c r="K5" s="8"/>
       <c r="L5" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="M5" s="8"/>
+    </row>
+    <row r="6" spans="1:25" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="M5" s="8"/>
-    </row>
-    <row r="6" spans="1:13" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>103</v>
-      </c>
       <c r="B6" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="8"/>
@@ -1492,19 +1625,19 @@
       </c>
       <c r="K6" s="8"/>
       <c r="L6" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M6" s="8"/>
     </row>
-    <row r="7" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>71</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>72</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="8"/>
@@ -1519,15 +1652,15 @@
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
-    <row r="8" spans="1:13" s="11" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" s="11" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>73</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>74</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="8"/>
@@ -1540,7 +1673,7 @@
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
     </row>
-    <row r="9" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>23</v>
       </c>
@@ -1553,10 +1686,10 @@
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>76</v>
       </c>
       <c r="H9" s="8"/>
       <c r="I9" s="8"/>
@@ -1567,9 +1700,9 @@
       <c r="L9" s="8"/>
       <c r="M9" s="8"/>
     </row>
-    <row r="10" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" s="11" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>27</v>
@@ -1590,30 +1723,46 @@
       <c r="L10" s="13"/>
       <c r="M10" s="8"/>
     </row>
-    <row r="11" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="1:25" s="11" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="8"/>
-    </row>
-    <row r="12" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="27"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="G11" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="29"/>
+      <c r="N11" s="29"/>
+      <c r="O11" s="29"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
+      <c r="R11" s="29"/>
+      <c r="S11" s="29"/>
+      <c r="T11" s="29"/>
+      <c r="U11" s="29"/>
+      <c r="V11" s="29"/>
+      <c r="W11" s="29"/>
+      <c r="X11" s="29"/>
+      <c r="Y11" s="29"/>
+    </row>
+    <row r="12" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>20</v>
       </c>
@@ -1636,7 +1785,7 @@
       <c r="L12" s="8"/>
       <c r="M12" s="8"/>
     </row>
-    <row r="13" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>20</v>
       </c>
@@ -1659,7 +1808,7 @@
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
     </row>
-    <row r="14" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>20</v>
       </c>
@@ -1682,15 +1831,15 @@
       <c r="L14" s="8"/>
       <c r="M14" s="8"/>
     </row>
-    <row r="15" spans="1:13" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" s="11" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="8"/>
@@ -1698,7 +1847,7 @@
       <c r="G15" s="10"/>
       <c r="H15" s="8"/>
       <c r="I15" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
@@ -1707,50 +1856,64 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8" t="s">
+    <row r="16" spans="1:25" s="11" customFormat="1" ht="69.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>239</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>240</v>
+      </c>
+      <c r="D16" s="27"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26" t="s">
+        <v>241</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="H16" s="26" t="s">
+        <v>243</v>
+      </c>
+      <c r="I16" s="26"/>
+      <c r="J16" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-    </row>
-    <row r="17" spans="1:13" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="29"/>
+      <c r="N16" s="29"/>
+      <c r="O16" s="29"/>
+      <c r="P16" s="29"/>
+      <c r="Q16" s="29"/>
+      <c r="R16" s="29"/>
+      <c r="S16" s="29"/>
+      <c r="T16" s="29"/>
+      <c r="U16" s="29"/>
+      <c r="V16" s="29"/>
+      <c r="W16" s="29"/>
+      <c r="X16" s="29"/>
+      <c r="Y16" s="29"/>
+    </row>
+    <row r="17" spans="1:25" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -1761,139 +1924,207 @@
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
     </row>
-    <row r="18" spans="1:13" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="10"/>
+      <c r="F18" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>84</v>
+      </c>
       <c r="H18" s="8"/>
-      <c r="I18" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="J18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8" t="s">
+        <v>9</v>
+      </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8"/>
-      <c r="M18" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="M18" s="8"/>
+    </row>
+    <row r="19" spans="1:25" s="11" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
       <c r="G19" s="10"/>
       <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="I19" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-    </row>
-    <row r="20" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="M19" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" s="11" customFormat="1" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>244</v>
+      </c>
+      <c r="C20" s="26" t="s">
+        <v>245</v>
+      </c>
+      <c r="D20" s="27"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="G20" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="H20" s="26" t="s">
+        <v>247</v>
+      </c>
+      <c r="I20" s="26"/>
+      <c r="J20" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="29"/>
+      <c r="S20" s="29"/>
+      <c r="T20" s="29"/>
+      <c r="U20" s="29"/>
+      <c r="V20" s="29"/>
+      <c r="W20" s="29"/>
+      <c r="X20" s="29"/>
+      <c r="Y20" s="29"/>
+    </row>
+    <row r="21" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="10"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-    </row>
-    <row r="21" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>68</v>
-      </c>
       <c r="B21" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D21" s="10"/>
-      <c r="E21" s="8" t="s">
-        <v>66</v>
-      </c>
+      <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="10"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
-      <c r="J21" s="8" t="s">
-        <v>9</v>
-      </c>
+      <c r="J21" s="8"/>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
     </row>
-    <row r="22" spans="1:13" s="6" customFormat="1" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
+    <row r="22" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="10"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+    </row>
+    <row r="23" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="10"/>
+      <c r="E23" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" s="8"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+    </row>
+    <row r="24" spans="1:25" s="6" customFormat="1" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="B22" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="D22" s="21"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-    </row>
-    <row r="23" spans="1:13" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
+      <c r="C24" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D24" s="21"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="22"/>
+    </row>
+    <row r="25" spans="1:25" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B25" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1922,13 +2153,13 @@
         <v>16</v>
       </c>
       <c r="D1" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>93</v>
-      </c>
       <c r="F1" s="16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1969,10 +2200,10 @@
         <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1980,10 +2211,10 @@
         <v>27</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1991,10 +2222,10 @@
         <v>27</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2002,10 +2233,10 @@
         <v>27</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2013,10 +2244,10 @@
         <v>27</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2024,10 +2255,10 @@
         <v>27</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2035,10 +2266,10 @@
         <v>27</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2046,10 +2277,10 @@
         <v>27</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -2057,10 +2288,10 @@
         <v>27</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -2068,10 +2299,10 @@
         <v>27</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2079,10 +2310,10 @@
         <v>27</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -2090,217 +2321,217 @@
         <v>27</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D25" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D28" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D29" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D30" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D31" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D32" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D34" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -2308,1626 +2539,1626 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E37" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E38" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E40" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E42" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E43" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E45" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E47" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E48" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E49" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E50" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E51" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E52" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E54" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E55" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E56" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E57" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E58" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E61" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E63" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E64" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E65" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E66" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E67" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E68" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E69" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E70" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E71" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E72" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E73" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E74" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E75" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E76" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E77" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E78" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E79" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E80" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E81" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E82" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E83" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E84" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E85" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E86" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E87" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E88" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E89" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E90" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E91" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E92" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E93" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F95" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F96" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F97" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F98" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F99" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F100" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F101" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F102" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F103" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F104" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F105" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F106" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F107" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F108" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F109" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F110" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F111" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F112" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F113" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F115" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F116" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F117" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F118" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F119" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F120" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F121" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F122" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F123" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F124" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F125" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F126" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F127" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F128" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F129" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F130" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F131" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F132" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F133" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F134" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F135" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F136" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F137" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F138" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F139" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F140" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F141" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F142" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F143" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F144" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F145" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F146" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B147" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F147" t="s">
         <v>217</v>
-      </c>
-      <c r="C147" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="F147" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F148" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F149" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F150" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F151" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F152" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -4863,10 +5094,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>19</v>

</xml_diff>